<commit_message>
Added grating levels ranging from 0.10 to 0.01 (and 0)
</commit_message>
<xml_diff>
--- a/Components_parameters.xlsx
+++ b/Components_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\recursos\H-IBL.Task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94320A05-6A49-4600-8181-1AEA57A93BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A479A15-9AD4-47AE-B211-CFA5E3B28E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="32">
   <si>
     <t>position</t>
   </si>
@@ -91,15 +91,6 @@
     <t>sin</t>
   </si>
   <si>
-    <t>(25, 0)</t>
-  </si>
-  <si>
-    <t>(-25, 0)</t>
-  </si>
-  <si>
-    <t>0.30</t>
-  </si>
-  <si>
     <t>mask</t>
   </si>
   <si>
@@ -119,6 +110,36 @@
   </si>
   <si>
     <t>(-35, 0)</t>
+  </si>
+  <si>
+    <t>0.10</t>
+  </si>
+  <si>
+    <t>0.0</t>
+  </si>
+  <si>
+    <t>0.05</t>
+  </si>
+  <si>
+    <t>0.09</t>
+  </si>
+  <si>
+    <t>0.07</t>
+  </si>
+  <si>
+    <t>0.06</t>
+  </si>
+  <si>
+    <t>0.04</t>
+  </si>
+  <si>
+    <t>0.03</t>
+  </si>
+  <si>
+    <t>0.02</t>
+  </si>
+  <si>
+    <t>0.01</t>
   </si>
 </sst>
 </file>
@@ -442,7 +463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="8" max="8" width="9.7109375" customWidth="1"/>
@@ -459,16 +480,16 @@
         <v>13</v>
       </c>
       <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" t="s">
-        <v>21</v>
-      </c>
       <c r="G1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
         <v>2</v>
@@ -488,16 +509,16 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
       </c>
       <c r="C2" t="s">
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -526,16 +547,16 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -564,16 +585,16 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -602,16 +623,16 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
         <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -640,16 +661,16 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
       </c>
       <c r="C6" t="s">
         <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E6">
         <v>3</v>
@@ -678,16 +699,16 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -716,16 +737,16 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
       </c>
       <c r="C8" t="s">
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E8">
         <v>3</v>
@@ -754,16 +775,16 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s">
         <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -792,16 +813,16 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
       </c>
       <c r="C10" t="s">
         <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -830,16 +851,16 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
         <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E11">
         <v>3</v>
@@ -868,16 +889,16 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12">
-        <v>1</v>
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>24</v>
       </c>
       <c r="C12" t="s">
         <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E12">
         <v>3</v>
@@ -906,16 +927,16 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
         <v>14</v>
       </c>
       <c r="D13" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E13">
         <v>3</v>
@@ -944,16 +965,16 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
+        <v>21</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
       </c>
       <c r="C14" t="s">
         <v>14</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E14">
         <v>3</v>
@@ -982,16 +1003,16 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="C15" t="s">
         <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E15">
         <v>3</v>
@@ -1020,16 +1041,16 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
       </c>
       <c r="C16" t="s">
         <v>14</v>
       </c>
       <c r="D16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E16">
         <v>3</v>
@@ -1058,16 +1079,16 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C17" t="s">
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E17">
         <v>3</v>
@@ -1096,16 +1117,16 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>30</v>
       </c>
       <c r="C18" t="s">
         <v>14</v>
       </c>
       <c r="D18" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E18">
         <v>3</v>
@@ -1134,16 +1155,16 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="C19" t="s">
         <v>14</v>
       </c>
       <c r="D19" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E19">
         <v>3</v>
@@ -1172,16 +1193,16 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>15</v>
-      </c>
-      <c r="B20">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B20" t="s">
+        <v>31</v>
       </c>
       <c r="C20" t="s">
         <v>14</v>
       </c>
       <c r="D20" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E20">
         <v>3</v>
@@ -1210,16 +1231,16 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="C21" t="s">
         <v>14</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E21">
         <v>3</v>
@@ -1248,16 +1269,16 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>23</v>
       </c>
       <c r="C22" t="s">
         <v>14</v>
       </c>
       <c r="D22" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E22">
         <v>3</v>
@@ -1286,16 +1307,16 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C23" t="s">
         <v>14</v>
       </c>
       <c r="D23" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E23">
         <v>3</v>
@@ -1324,16 +1345,16 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B24">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>22</v>
       </c>
       <c r="C24" t="s">
         <v>14</v>
       </c>
       <c r="D24" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E24">
         <v>3</v>
@@ -1362,16 +1383,16 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B25" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C25" t="s">
         <v>14</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E25">
         <v>3</v>
@@ -1400,16 +1421,16 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>15</v>
-      </c>
-      <c r="B26">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B26" t="s">
+        <v>25</v>
       </c>
       <c r="C26" t="s">
         <v>14</v>
       </c>
       <c r="D26" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E26">
         <v>3</v>
@@ -1438,16 +1459,16 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C27" t="s">
         <v>14</v>
       </c>
       <c r="D27" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E27">
         <v>3</v>
@@ -1476,16 +1497,16 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>15</v>
-      </c>
-      <c r="B28">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B28" t="s">
+        <v>11</v>
       </c>
       <c r="C28" t="s">
         <v>14</v>
       </c>
       <c r="D28" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E28">
         <v>3</v>
@@ -1514,16 +1535,16 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C29" t="s">
         <v>14</v>
       </c>
       <c r="D29" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E29">
         <v>3</v>
@@ -1552,16 +1573,16 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B30" t="s">
+        <v>26</v>
       </c>
       <c r="C30" t="s">
         <v>14</v>
       </c>
       <c r="D30" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E30">
         <v>3</v>
@@ -1590,16 +1611,16 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B31" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="C31" t="s">
         <v>14</v>
       </c>
       <c r="D31" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E31">
         <v>3</v>
@@ -1628,16 +1649,16 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>15</v>
-      </c>
-      <c r="B32">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B32" t="s">
+        <v>27</v>
       </c>
       <c r="C32" t="s">
         <v>14</v>
       </c>
       <c r="D32" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E32">
         <v>3</v>
@@ -1666,16 +1687,16 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B33" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="C33" t="s">
         <v>14</v>
       </c>
       <c r="D33" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E33">
         <v>3</v>
@@ -1704,16 +1725,16 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>15</v>
-      </c>
-      <c r="B34">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B34" t="s">
+        <v>24</v>
       </c>
       <c r="C34" t="s">
         <v>14</v>
       </c>
       <c r="D34" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E34">
         <v>3</v>
@@ -1742,16 +1763,16 @@
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B35" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C35" t="s">
         <v>14</v>
       </c>
       <c r="D35" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E35">
         <v>3</v>
@@ -1780,16 +1801,16 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>15</v>
-      </c>
-      <c r="B36">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B36" t="s">
+        <v>28</v>
       </c>
       <c r="C36" t="s">
         <v>14</v>
       </c>
       <c r="D36" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E36">
         <v>3</v>
@@ -1818,16 +1839,16 @@
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B37" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="C37" t="s">
         <v>14</v>
       </c>
       <c r="D37" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E37">
         <v>3</v>
@@ -1856,16 +1877,16 @@
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>15</v>
-      </c>
-      <c r="B38">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B38" t="s">
+        <v>29</v>
       </c>
       <c r="C38" t="s">
         <v>14</v>
       </c>
       <c r="D38" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E38">
         <v>3</v>
@@ -1894,16 +1915,16 @@
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B39" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C39" t="s">
         <v>14</v>
       </c>
       <c r="D39" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E39">
         <v>3</v>
@@ -1932,16 +1953,16 @@
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>15</v>
-      </c>
-      <c r="B40">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="B40" t="s">
+        <v>30</v>
       </c>
       <c r="C40" t="s">
         <v>14</v>
       </c>
       <c r="D40" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E40">
         <v>3</v>
@@ -1970,16 +1991,16 @@
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B41" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="C41" t="s">
         <v>14</v>
       </c>
       <c r="D41" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E41">
         <v>3</v>
@@ -2003,6 +2024,158 @@
         <v>12</v>
       </c>
       <c r="O41" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>21</v>
+      </c>
+      <c r="B42" t="s">
+        <v>31</v>
+      </c>
+      <c r="C42" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" t="s">
+        <v>16</v>
+      </c>
+      <c r="E42">
+        <v>3</v>
+      </c>
+      <c r="F42">
+        <v>1</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42" t="s">
+        <v>6</v>
+      </c>
+      <c r="I42" t="s">
+        <v>5</v>
+      </c>
+      <c r="M42" t="s">
+        <v>10</v>
+      </c>
+      <c r="N42" t="s">
+        <v>12</v>
+      </c>
+      <c r="O42" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>20</v>
+      </c>
+      <c r="B43" t="s">
+        <v>31</v>
+      </c>
+      <c r="C43" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43" t="s">
+        <v>16</v>
+      </c>
+      <c r="E43">
+        <v>3</v>
+      </c>
+      <c r="F43">
+        <v>1</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43" t="s">
+        <v>6</v>
+      </c>
+      <c r="I43" t="s">
+        <v>4</v>
+      </c>
+      <c r="M43" t="s">
+        <v>10</v>
+      </c>
+      <c r="N43" t="s">
+        <v>12</v>
+      </c>
+      <c r="O43" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>21</v>
+      </c>
+      <c r="B44" t="s">
+        <v>23</v>
+      </c>
+      <c r="C44" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44" t="s">
+        <v>16</v>
+      </c>
+      <c r="E44">
+        <v>3</v>
+      </c>
+      <c r="F44">
+        <v>1</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44" t="s">
+        <v>6</v>
+      </c>
+      <c r="I44" t="s">
+        <v>5</v>
+      </c>
+      <c r="M44" t="s">
+        <v>10</v>
+      </c>
+      <c r="N44" t="s">
+        <v>12</v>
+      </c>
+      <c r="O44" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" t="s">
+        <v>23</v>
+      </c>
+      <c r="C45" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" t="s">
+        <v>16</v>
+      </c>
+      <c r="E45">
+        <v>3</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45" t="s">
+        <v>6</v>
+      </c>
+      <c r="I45" t="s">
+        <v>4</v>
+      </c>
+      <c r="M45" t="s">
+        <v>10</v>
+      </c>
+      <c r="N45" t="s">
+        <v>12</v>
+      </c>
+      <c r="O45" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reverted to key response only version
</commit_message>
<xml_diff>
--- a/Components_parameters.xlsx
+++ b/Components_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\recursos\H-IBL.Task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC6FC21F-9AD7-4B19-A3B9-8FF6F49A08FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6FAA5A-816E-449A-BBF0-03993CF3FD10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19005" yWindow="1575" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
remove bar completion code from the trial itself
</commit_message>
<xml_diff>
--- a/Components_parameters.xlsx
+++ b/Components_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\recursos\H-IBL.Task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA6FAA5A-816E-449A-BBF0-03993CF3FD10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E261B44C-95B2-424D-AB94-FCFEF8F32194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -94,12 +94,6 @@
     <t>orientation</t>
   </si>
   <si>
-    <t>(35, 0)</t>
-  </si>
-  <si>
-    <t>(-35, 0)</t>
-  </si>
-  <si>
     <t>0.10</t>
   </si>
   <si>
@@ -131,6 +125,12 @@
   </si>
   <si>
     <t>gauss</t>
+  </si>
+  <si>
+    <t>(15, 0)</t>
+  </si>
+  <si>
+    <t>(-15, 0)</t>
   </si>
 </sst>
 </file>
@@ -497,16 +497,16 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
       <c r="C2" t="s">
         <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -532,16 +532,16 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
       <c r="C3" t="s">
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -567,16 +567,16 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -602,16 +602,16 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -637,7 +637,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -646,7 +646,7 @@
         <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E6">
         <v>3</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
@@ -681,7 +681,7 @@
         <v>11</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -707,16 +707,16 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E8">
         <v>3</v>
@@ -742,16 +742,16 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -777,16 +777,16 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
         <v>11</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -812,16 +812,16 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E11">
         <v>3</v>
@@ -847,16 +847,16 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C12" t="s">
         <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E12">
         <v>3</v>
@@ -882,16 +882,16 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C13" t="s">
         <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E13">
         <v>3</v>
@@ -917,16 +917,16 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C14" t="s">
         <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E14">
         <v>3</v>
@@ -952,16 +952,16 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C15" t="s">
         <v>11</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E15">
         <v>3</v>
@@ -987,16 +987,16 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C16" t="s">
         <v>11</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E16">
         <v>3</v>
@@ -1022,16 +1022,16 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
         <v>11</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E17">
         <v>3</v>
@@ -1057,16 +1057,16 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C18" t="s">
         <v>11</v>
       </c>
       <c r="D18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E18">
         <v>3</v>
@@ -1092,16 +1092,16 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C19" t="s">
         <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E19">
         <v>3</v>
@@ -1127,16 +1127,16 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
         <v>11</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E20">
         <v>3</v>
@@ -1162,16 +1162,16 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C21" t="s">
         <v>11</v>
       </c>
       <c r="D21" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E21">
         <v>3</v>
@@ -1197,16 +1197,16 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C22" t="s">
         <v>11</v>
       </c>
       <c r="D22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E22">
         <v>3</v>
@@ -1232,16 +1232,16 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" t="s">
         <v>17</v>
       </c>
-      <c r="B23" t="s">
-        <v>19</v>
-      </c>
       <c r="C23" t="s">
         <v>11</v>
       </c>
       <c r="D23" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E23">
         <v>3</v>
@@ -1267,16 +1267,16 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
         <v>16</v>
       </c>
-      <c r="B24" t="s">
-        <v>18</v>
-      </c>
       <c r="C24" t="s">
         <v>11</v>
       </c>
       <c r="D24" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E24">
         <v>3</v>
@@ -1302,16 +1302,16 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C25" t="s">
         <v>11</v>
       </c>
       <c r="D25" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E25">
         <v>3</v>
@@ -1337,16 +1337,16 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C26" t="s">
         <v>11</v>
       </c>
       <c r="D26" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E26">
         <v>3</v>
@@ -1372,16 +1372,16 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C27" t="s">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E27">
         <v>3</v>
@@ -1407,7 +1407,7 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B28" t="s">
         <v>8</v>
@@ -1416,7 +1416,7 @@
         <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E28">
         <v>3</v>
@@ -1442,7 +1442,7 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s">
         <v>8</v>
@@ -1451,7 +1451,7 @@
         <v>11</v>
       </c>
       <c r="D29" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E29">
         <v>3</v>
@@ -1477,16 +1477,16 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B30" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C30" t="s">
         <v>11</v>
       </c>
       <c r="D30" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E30">
         <v>3</v>
@@ -1512,16 +1512,16 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B31" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C31" t="s">
         <v>11</v>
       </c>
       <c r="D31" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E31">
         <v>3</v>
@@ -1547,16 +1547,16 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B32" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C32" t="s">
         <v>11</v>
       </c>
       <c r="D32" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E32">
         <v>3</v>
@@ -1582,16 +1582,16 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B33" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C33" t="s">
         <v>11</v>
       </c>
       <c r="D33" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E33">
         <v>3</v>
@@ -1617,16 +1617,16 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B34" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C34" t="s">
         <v>11</v>
       </c>
       <c r="D34" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E34">
         <v>3</v>
@@ -1652,16 +1652,16 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B35" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C35" t="s">
         <v>11</v>
       </c>
       <c r="D35" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E35">
         <v>3</v>
@@ -1687,16 +1687,16 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B36" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C36" t="s">
         <v>11</v>
       </c>
       <c r="D36" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E36">
         <v>3</v>
@@ -1722,16 +1722,16 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B37" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C37" t="s">
         <v>11</v>
       </c>
       <c r="D37" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E37">
         <v>3</v>
@@ -1757,16 +1757,16 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B38" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C38" t="s">
         <v>11</v>
       </c>
       <c r="D38" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E38">
         <v>3</v>
@@ -1792,16 +1792,16 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B39" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C39" t="s">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E39">
         <v>3</v>
@@ -1827,16 +1827,16 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B40" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C40" t="s">
         <v>11</v>
       </c>
       <c r="D40" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E40">
         <v>3</v>
@@ -1862,16 +1862,16 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B41" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C41" t="s">
         <v>11</v>
       </c>
       <c r="D41" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E41">
         <v>3</v>
@@ -1897,16 +1897,16 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B42" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C42" t="s">
         <v>11</v>
       </c>
       <c r="D42" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E42">
         <v>3</v>
@@ -1932,16 +1932,16 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B43" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C43" t="s">
         <v>11</v>
       </c>
       <c r="D43" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E43">
         <v>3</v>
@@ -1967,16 +1967,16 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>28</v>
+      </c>
+      <c r="B44" t="s">
         <v>17</v>
       </c>
-      <c r="B44" t="s">
-        <v>19</v>
-      </c>
       <c r="C44" t="s">
         <v>11</v>
       </c>
       <c r="D44" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E44">
         <v>3</v>
@@ -2002,16 +2002,16 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B45" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C45" t="s">
         <v>11</v>
       </c>
       <c r="D45" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E45">
         <v>3</v>

</xml_diff>